<commit_message>
fix: Optimize matching rules in invoice generator for precise label matching
</commit_message>
<xml_diff>
--- a/vba/报关合同模板.xlsx
+++ b/vba/报关合同模板.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="13160"/>
+    <workbookView windowWidth="28800" windowHeight="13660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -919,7 +919,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="31" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="31" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="31" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="B13" s="8">
-        <v>44196</v>
+        <v>46387</v>
       </c>
       <c r="C13" s="8"/>
       <c r="D13" s="9" t="s">

</xml_diff>